<commit_message>
Output Excel and png of Updated POST API /api/contact_us response body (#1)
</commit_message>
<xml_diff>
--- a/api_task_contact_us/src/Outputs/Excel_Outputs/Contact_us_Excel_Sheet_Apis/Codolog_Contact_Us_GET_POST_API's_Assignment.xlsx
+++ b/api_task_contact_us/src/Outputs/Excel_Outputs/Contact_us_Excel_Sheet_Apis/Codolog_Contact_Us_GET_POST_API's_Assignment.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bappi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dump\Codolog\Spring\Apis\Git_contact_us\Codolog_Spring_Codes\api_task_contact_us\src\Outputs\Excel_Outputs\Contact_us_Excel_Sheet_Apis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5281EC15-BC2D-48D0-A379-20F83B346E9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4C11B7F-A5AD-48DC-B1B5-D45B88B8192E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{861E19F2-D9EC-49AA-A329-F460E9A92DF9}"/>
   </bookViews>
@@ -68,19 +68,6 @@
     <t>GET</t>
   </si>
   <si>
-    <t>[
-    {
-        "contactno": 9324779110,
-        "createdAt": "2026-04-16T23:02:59.857921",
-        "email": "bappi@gmail.com",
-        "fullname": "Bappi Singh",
-        "id": 1,
-        "message": "Hello, i would like to connect with mentor !!! ",
-        "subject": "Enquiry Test"
-    }
-]</t>
-  </si>
-  <si>
     <t>postman request 'http://localhost:8082/api/contact/all' \
   --body ''</t>
   </si>
@@ -91,38 +78,71 @@
     <t>POST</t>
   </si>
   <si>
+    <t>null</t>
+  </si>
+  <si>
+    <t>{
+    "fullname": "Sujal Atak",
+    "email": "sujal@gmail.com",
+    "contactno": "9012345678",
+    "subject": "Course Inquiry",
+    "message": "Good afternoon, I want to know more about the advanced Java training program !"
+}</t>
+  </si>
+  <si>
+    <t>{
+    "status": 201,
+    "message": "Data inserted successfully!",
+    "data": null,
+    "timestamp": "2026-04-24T17:37:03.6203402"
+}</t>
+  </si>
+  <si>
     <t>postman request POST 'http://localhost:8082/api/contact/submit' \
-  --header 'Content-Type: application/json' \
   --body '{
-    "fullname": "Bappi Singh",
-    "email": "bappi@gmail.com",
-    "contactno": "9324779110",
-    "subject": "Enquiry Test",
-    "message": "Hello, i would like to connect with mentor !!! "
-}'</t>
+    "fullname": "Sujal Atak",
+    "email": "sujal@gmail.com",
+    "contactno": "9012345678",
+    "subject": "Course Inquiry",
+    "message": "Good afternoon, I want to know more about the advanced Java training program !"
+}
+'</t>
   </si>
   <si>
     <t>{
-    "fullname": "Bappi Singh",
-    "email": "bappi@gmail.com",
-    "contactno": "9324779110",
-    "subject": "Enquiry Test",
-    "message": "Hello, i would like to connect with mentor !!! "
+    "status": 200,
+    "message": "Messages fetched successfully",
+    "data": [
+        {
+            "contactno": 9324779110,
+            "createdAt": "2026-04-16T23:02:59.857921",
+            "email": "bappi@gmail.com",
+            "fullname": "Bappi Singh",
+            "id": 1,
+            "message": "Hello, i would like to connect with mentor !!! ",
+            "subject": "Enquiry Test"
+        },
+        {
+            "contactno": 9876543210,
+            "createdAt": "2026-04-24T17:07:02.288588",
+            "email": "riya@gmail.com",
+            "fullname": "Riya Mehta",
+            "id": 3,
+            "message": "Hi, I am interested in joining your upcoming workshop !",
+            "subject": "Mentorship Request"
+        },
+        {
+            "contactno": 9012345678,
+            "createdAt": "2026-04-24T17:37:03.561316",
+            "email": "sujal@gmail.com",
+            "fullname": "Sujal Atak",
+            "id": 4,
+            "message": "Good afternoon, I want to know more about the advanced Java training program !",
+            "subject": "Course Inquiry"
+        }
+    ],
+    "timestamp": "2026-04-24T17:37:26.3003391"
 }</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> {
-        "contactno": 9324779110,
-        "createdAt": "2026-04-16T23:02:59.857921",
-        "email": "bappi@gmail.com",
-        "fullname": "Bappi Singh",
-        "id": 1,
-        "message": "Hello, i would like to connect with mentor !!! ",
-        "subject": "Enquiry Test"
-    }</t>
-  </si>
-  <si>
-    <t>null</t>
   </si>
 </sst>
 </file>
@@ -533,8 +553,8 @@
     <col min="3" max="3" width="39.73046875" customWidth="1"/>
     <col min="4" max="4" width="17.86328125" customWidth="1"/>
     <col min="5" max="5" width="24.6640625" customWidth="1"/>
-    <col min="6" max="6" width="38.19921875" customWidth="1"/>
-    <col min="7" max="7" width="26.1328125" customWidth="1"/>
+    <col min="6" max="6" width="50.1328125" customWidth="1"/>
+    <col min="7" max="7" width="32.9296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
@@ -560,7 +580,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="185.65" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:7" ht="199.9" x14ac:dyDescent="0.5">
       <c r="A2">
         <v>1</v>
       </c>
@@ -568,22 +588,22 @@
         <v>7</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
         <v>12</v>
       </c>
-      <c r="D2" t="s">
-        <v>13</v>
-      </c>
       <c r="E2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>14</v>
-      </c>
     </row>
-    <row r="3" spans="1:7" ht="187.15" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:7" ht="409.6" x14ac:dyDescent="0.7">
       <c r="A3">
         <v>2</v>
       </c>
@@ -597,13 +617,13 @@
         <v>9</v>
       </c>
       <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>10</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>